<commit_message>
Add v6 assessment content and scoring updates
</commit_message>
<xml_diff>
--- a/public/downloads/LJ3_HV_OpenData.xlsx
+++ b/public/downloads/LJ3_HV_OpenData.xlsx
@@ -1,82 +1,433 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Energie" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Energie'!A1:E71</definedName>
+  </definedNames>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
   <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E71"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H71"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Jaar</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Woningtype</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Verbruik</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Kosten</t>
-        </is>
+      <c r="A1" t="str">
+        <v>Code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Jaar</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Woningtype</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Verbruik</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Kosten</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>E13</t>
-        </is>
+      <c r="A2" t="str">
+        <v>E13</v>
       </c>
       <c r="B2">
         <v>2024</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C2" t="str">
+        <v>A</v>
       </c>
       <c r="D2">
         <v>1600</v>
@@ -84,20 +435,22 @@
       <c r="E2">
         <v>999</v>
       </c>
+      <c r="F2" t="str">
+        <v>Tip: gebruik SOM.ALS om totale Kosten voor Woningtype A te berekenen. Typ alleen de uitkomst in cel H2.</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>E02</t>
-        </is>
+      <c r="A3" t="str">
+        <v>E02</v>
       </c>
       <c r="B3">
         <v>2028</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C3" t="str">
+        <v>B</v>
       </c>
       <c r="D3">
         <v>1180</v>
@@ -107,18 +460,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>E06</t>
-        </is>
+      <c r="A4" t="str">
+        <v>E06</v>
       </c>
       <c r="B4">
         <v>2025</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C4" t="str">
+        <v>A</v>
       </c>
       <c r="D4">
         <v>1400</v>
@@ -128,18 +477,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>E20</t>
-        </is>
+      <c r="A5" t="str">
+        <v>E20</v>
       </c>
       <c r="B5">
         <v>2011</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C5" t="str">
+        <v>A</v>
       </c>
       <c r="D5">
         <v>850</v>
@@ -149,18 +494,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>E21</t>
-        </is>
+      <c r="A6" t="str">
+        <v>E21</v>
       </c>
       <c r="B6">
         <v>2011</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C6" t="str">
+        <v>B</v>
       </c>
       <c r="D6">
         <v>923</v>
@@ -170,18 +511,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>E22</t>
-        </is>
+      <c r="A7" t="str">
+        <v>E22</v>
       </c>
       <c r="B7">
         <v>2013</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C7" t="str">
+        <v>C</v>
       </c>
       <c r="D7">
         <v>996</v>
@@ -191,18 +528,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>E23</t>
-        </is>
+      <c r="A8" t="str">
+        <v>E23</v>
       </c>
       <c r="B8">
         <v>2014</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C8" t="str">
+        <v>D</v>
       </c>
       <c r="D8">
         <v>1069</v>
@@ -212,18 +545,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>E24</t>
-        </is>
+      <c r="A9" t="str">
+        <v>E24</v>
       </c>
       <c r="B9">
         <v>2015</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C9" t="str">
+        <v>A</v>
       </c>
       <c r="D9">
         <v>1142</v>
@@ -233,18 +562,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>E25</t>
-        </is>
+      <c r="A10" t="str">
+        <v>E25</v>
       </c>
       <c r="B10">
         <v>2015</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C10" t="str">
+        <v>B</v>
       </c>
       <c r="D10">
         <v>1215</v>
@@ -254,18 +579,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>E26</t>
-        </is>
+      <c r="A11" t="str">
+        <v>E26</v>
       </c>
       <c r="B11">
         <v>2017</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C11" t="str">
+        <v>C</v>
       </c>
       <c r="D11">
         <v>1288</v>
@@ -275,18 +596,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>E27</t>
-        </is>
+      <c r="A12" t="str">
+        <v>E27</v>
       </c>
       <c r="B12">
         <v>2018</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C12" t="str">
+        <v>D</v>
       </c>
       <c r="D12">
         <v>1361</v>
@@ -296,18 +613,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>E28</t>
-        </is>
+      <c r="A13" t="str">
+        <v>E28</v>
       </c>
       <c r="B13">
         <v>2019</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C13" t="str">
+        <v>A</v>
       </c>
       <c r="D13">
         <v>1434</v>
@@ -317,18 +630,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E29</t>
-        </is>
+      <c r="A14" t="str">
+        <v>E29</v>
       </c>
       <c r="B14">
         <v>2019</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C14" t="str">
+        <v>B</v>
       </c>
       <c r="D14">
         <v>1507</v>
@@ -338,18 +647,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>E30</t>
-        </is>
+      <c r="A15" t="str">
+        <v>E30</v>
       </c>
       <c r="B15">
         <v>2021</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C15" t="str">
+        <v>C</v>
       </c>
       <c r="D15">
         <v>1580</v>
@@ -359,18 +664,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>E31</t>
-        </is>
+      <c r="A16" t="str">
+        <v>E31</v>
       </c>
       <c r="B16">
         <v>2022</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C16" t="str">
+        <v>D</v>
       </c>
       <c r="D16">
         <v>1653</v>
@@ -380,18 +681,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>E32</t>
-        </is>
+      <c r="A17" t="str">
+        <v>E32</v>
       </c>
       <c r="B17">
         <v>2023</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C17" t="str">
+        <v>A</v>
       </c>
       <c r="D17">
         <v>1726</v>
@@ -401,18 +698,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>E33</t>
-        </is>
+      <c r="A18" t="str">
+        <v>E33</v>
       </c>
       <c r="B18">
         <v>2023</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C18" t="str">
+        <v>B</v>
       </c>
       <c r="D18">
         <v>899</v>
@@ -422,18 +715,14 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>E34</t>
-        </is>
+      <c r="A19" t="str">
+        <v>E34</v>
       </c>
       <c r="B19">
         <v>2025</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C19" t="str">
+        <v>C</v>
       </c>
       <c r="D19">
         <v>972</v>
@@ -443,18 +732,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>E35</t>
-        </is>
+      <c r="A20" t="str">
+        <v>E35</v>
       </c>
       <c r="B20">
         <v>2026</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C20" t="str">
+        <v>D</v>
       </c>
       <c r="D20">
         <v>1045</v>
@@ -464,18 +749,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>E36</t>
-        </is>
+      <c r="A21" t="str">
+        <v>E36</v>
       </c>
       <c r="B21">
         <v>2027</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C21" t="str">
+        <v>A</v>
       </c>
       <c r="D21">
         <v>1118</v>
@@ -485,18 +766,14 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>E37</t>
-        </is>
+      <c r="A22" t="str">
+        <v>E37</v>
       </c>
       <c r="B22">
         <v>2010</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C22" t="str">
+        <v>B</v>
       </c>
       <c r="D22">
         <v>1191</v>
@@ -506,18 +783,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>E38</t>
-        </is>
+      <c r="A23" t="str">
+        <v>E38</v>
       </c>
       <c r="B23">
         <v>2012</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C23" t="str">
+        <v>C</v>
       </c>
       <c r="D23">
         <v>1264</v>
@@ -527,18 +800,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>E39</t>
-        </is>
+      <c r="A24" t="str">
+        <v>E39</v>
       </c>
       <c r="B24">
         <v>2013</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C24" t="str">
+        <v>D</v>
       </c>
       <c r="D24">
         <v>1337</v>
@@ -548,18 +817,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>E40</t>
-        </is>
+      <c r="A25" t="str">
+        <v>E40</v>
       </c>
       <c r="B25">
         <v>2014</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C25" t="str">
+        <v>A</v>
       </c>
       <c r="D25">
         <v>1410</v>
@@ -569,18 +834,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>E41</t>
-        </is>
+      <c r="A26" t="str">
+        <v>E41</v>
       </c>
       <c r="B26">
         <v>2014</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C26" t="str">
+        <v>B</v>
       </c>
       <c r="D26">
         <v>1483</v>
@@ -590,18 +851,14 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>E42</t>
-        </is>
+      <c r="A27" t="str">
+        <v>E42</v>
       </c>
       <c r="B27">
         <v>2016</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C27" t="str">
+        <v>C</v>
       </c>
       <c r="D27">
         <v>1556</v>
@@ -611,18 +868,14 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>E43</t>
-        </is>
+      <c r="A28" t="str">
+        <v>E43</v>
       </c>
       <c r="B28">
         <v>2017</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C28" t="str">
+        <v>D</v>
       </c>
       <c r="D28">
         <v>1629</v>
@@ -632,18 +885,14 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E44</t>
-        </is>
+      <c r="A29" t="str">
+        <v>E44</v>
       </c>
       <c r="B29">
         <v>2018</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C29" t="str">
+        <v>A</v>
       </c>
       <c r="D29">
         <v>1702</v>
@@ -653,18 +902,14 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>E45</t>
-        </is>
+      <c r="A30" t="str">
+        <v>E45</v>
       </c>
       <c r="B30">
         <v>2018</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C30" t="str">
+        <v>B</v>
       </c>
       <c r="D30">
         <v>875</v>
@@ -674,18 +919,14 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>E46</t>
-        </is>
+      <c r="A31" t="str">
+        <v>E46</v>
       </c>
       <c r="B31">
         <v>2020</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C31" t="str">
+        <v>C</v>
       </c>
       <c r="D31">
         <v>948</v>
@@ -695,18 +936,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>E47</t>
-        </is>
+      <c r="A32" t="str">
+        <v>E47</v>
       </c>
       <c r="B32">
         <v>2021</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C32" t="str">
+        <v>D</v>
       </c>
       <c r="D32">
         <v>1021</v>
@@ -716,18 +953,14 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>E48</t>
-        </is>
+      <c r="A33" t="str">
+        <v>E48</v>
       </c>
       <c r="B33">
         <v>2022</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C33" t="str">
+        <v>A</v>
       </c>
       <c r="D33">
         <v>1094</v>
@@ -737,18 +970,14 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>E49</t>
-        </is>
+      <c r="A34" t="str">
+        <v>E49</v>
       </c>
       <c r="B34">
         <v>2022</v>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C34" t="str">
+        <v>B</v>
       </c>
       <c r="D34">
         <v>1167</v>
@@ -758,18 +987,14 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>E50</t>
-        </is>
+      <c r="A35" t="str">
+        <v>E50</v>
       </c>
       <c r="B35">
         <v>2024</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C35" t="str">
+        <v>C</v>
       </c>
       <c r="D35">
         <v>1240</v>
@@ -779,18 +1004,14 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>E51</t>
-        </is>
+      <c r="A36" t="str">
+        <v>E51</v>
       </c>
       <c r="B36">
         <v>2025</v>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C36" t="str">
+        <v>D</v>
       </c>
       <c r="D36">
         <v>1313</v>
@@ -800,18 +1021,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>E52</t>
-        </is>
+      <c r="A37" t="str">
+        <v>E52</v>
       </c>
       <c r="B37">
         <v>2026</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C37" t="str">
+        <v>A</v>
       </c>
       <c r="D37">
         <v>1386</v>
@@ -821,18 +1038,14 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>E53</t>
-        </is>
+      <c r="A38" t="str">
+        <v>E53</v>
       </c>
       <c r="B38">
         <v>2026</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C38" t="str">
+        <v>B</v>
       </c>
       <c r="D38">
         <v>1459</v>
@@ -842,18 +1055,14 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>E54</t>
-        </is>
+      <c r="A39" t="str">
+        <v>E54</v>
       </c>
       <c r="B39">
         <v>2011</v>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C39" t="str">
+        <v>C</v>
       </c>
       <c r="D39">
         <v>1532</v>
@@ -863,18 +1072,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>E55</t>
-        </is>
+      <c r="A40" t="str">
+        <v>E55</v>
       </c>
       <c r="B40">
         <v>2012</v>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C40" t="str">
+        <v>D</v>
       </c>
       <c r="D40">
         <v>1605</v>
@@ -884,18 +1089,14 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>E56</t>
-        </is>
+      <c r="A41" t="str">
+        <v>E56</v>
       </c>
       <c r="B41">
         <v>2013</v>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C41" t="str">
+        <v>A</v>
       </c>
       <c r="D41">
         <v>1678</v>
@@ -905,18 +1106,14 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>E57</t>
-        </is>
+      <c r="A42" t="str">
+        <v>E57</v>
       </c>
       <c r="B42">
         <v>2013</v>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C42" t="str">
+        <v>B</v>
       </c>
       <c r="D42">
         <v>851</v>
@@ -926,18 +1123,14 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>E58</t>
-        </is>
+      <c r="A43" t="str">
+        <v>E58</v>
       </c>
       <c r="B43">
         <v>2015</v>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C43" t="str">
+        <v>C</v>
       </c>
       <c r="D43">
         <v>924</v>
@@ -947,18 +1140,14 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>E59</t>
-        </is>
+      <c r="A44" t="str">
+        <v>E59</v>
       </c>
       <c r="B44">
         <v>2016</v>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C44" t="str">
+        <v>D</v>
       </c>
       <c r="D44">
         <v>997</v>
@@ -968,18 +1157,14 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>E60</t>
-        </is>
+      <c r="A45" t="str">
+        <v>E60</v>
       </c>
       <c r="B45">
         <v>2017</v>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C45" t="str">
+        <v>A</v>
       </c>
       <c r="D45">
         <v>1070</v>
@@ -989,18 +1174,14 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>E61</t>
-        </is>
+      <c r="A46" t="str">
+        <v>E61</v>
       </c>
       <c r="B46">
         <v>2017</v>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C46" t="str">
+        <v>B</v>
       </c>
       <c r="D46">
         <v>1143</v>
@@ -1010,18 +1191,14 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>E62</t>
-        </is>
+      <c r="A47" t="str">
+        <v>E62</v>
       </c>
       <c r="B47">
         <v>2019</v>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C47" t="str">
+        <v>C</v>
       </c>
       <c r="D47">
         <v>1216</v>
@@ -1031,18 +1208,14 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>E63</t>
-        </is>
+      <c r="A48" t="str">
+        <v>E63</v>
       </c>
       <c r="B48">
         <v>2020</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C48" t="str">
+        <v>D</v>
       </c>
       <c r="D48">
         <v>1289</v>
@@ -1052,18 +1225,14 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>E64</t>
-        </is>
+      <c r="A49" t="str">
+        <v>E64</v>
       </c>
       <c r="B49">
         <v>2021</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C49" t="str">
+        <v>A</v>
       </c>
       <c r="D49">
         <v>1362</v>
@@ -1073,18 +1242,14 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>E65</t>
-        </is>
+      <c r="A50" t="str">
+        <v>E65</v>
       </c>
       <c r="B50">
         <v>2021</v>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C50" t="str">
+        <v>B</v>
       </c>
       <c r="D50">
         <v>1435</v>
@@ -1094,18 +1259,14 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>E66</t>
-        </is>
+      <c r="A51" t="str">
+        <v>E66</v>
       </c>
       <c r="B51">
         <v>2023</v>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C51" t="str">
+        <v>C</v>
       </c>
       <c r="D51">
         <v>1508</v>
@@ -1115,18 +1276,14 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>E67</t>
-        </is>
+      <c r="A52" t="str">
+        <v>E67</v>
       </c>
       <c r="B52">
         <v>2024</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C52" t="str">
+        <v>D</v>
       </c>
       <c r="D52">
         <v>1581</v>
@@ -1136,18 +1293,14 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>E68</t>
-        </is>
+      <c r="A53" t="str">
+        <v>E68</v>
       </c>
       <c r="B53">
         <v>2025</v>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C53" t="str">
+        <v>A</v>
       </c>
       <c r="D53">
         <v>1654</v>
@@ -1157,18 +1310,14 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>E69</t>
-        </is>
+      <c r="A54" t="str">
+        <v>E69</v>
       </c>
       <c r="B54">
         <v>2025</v>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C54" t="str">
+        <v>B</v>
       </c>
       <c r="D54">
         <v>1727</v>
@@ -1178,18 +1327,14 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>E70</t>
-        </is>
+      <c r="A55" t="str">
+        <v>E70</v>
       </c>
       <c r="B55">
         <v>2027</v>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C55" t="str">
+        <v>C</v>
       </c>
       <c r="D55">
         <v>900</v>
@@ -1199,18 +1344,14 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>E71</t>
-        </is>
+      <c r="A56" t="str">
+        <v>E71</v>
       </c>
       <c r="B56">
         <v>2011</v>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C56" t="str">
+        <v>D</v>
       </c>
       <c r="D56">
         <v>973</v>
@@ -1220,18 +1361,14 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>E72</t>
-        </is>
+      <c r="A57" t="str">
+        <v>E72</v>
       </c>
       <c r="B57">
         <v>2012</v>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C57" t="str">
+        <v>A</v>
       </c>
       <c r="D57">
         <v>1046</v>
@@ -1241,18 +1378,14 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>E73</t>
-        </is>
+      <c r="A58" t="str">
+        <v>E73</v>
       </c>
       <c r="B58">
         <v>2012</v>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C58" t="str">
+        <v>B</v>
       </c>
       <c r="D58">
         <v>1119</v>
@@ -1262,18 +1395,14 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>E74</t>
-        </is>
+      <c r="A59" t="str">
+        <v>E74</v>
       </c>
       <c r="B59">
         <v>2014</v>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C59" t="str">
+        <v>C</v>
       </c>
       <c r="D59">
         <v>1192</v>
@@ -1283,18 +1412,14 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>E75</t>
-        </is>
+      <c r="A60" t="str">
+        <v>E75</v>
       </c>
       <c r="B60">
         <v>2015</v>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C60" t="str">
+        <v>D</v>
       </c>
       <c r="D60">
         <v>1265</v>
@@ -1304,18 +1429,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>E76</t>
-        </is>
+      <c r="A61" t="str">
+        <v>E76</v>
       </c>
       <c r="B61">
         <v>2016</v>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C61" t="str">
+        <v>A</v>
       </c>
       <c r="D61">
         <v>1338</v>
@@ -1325,18 +1446,14 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>E77</t>
-        </is>
+      <c r="A62" t="str">
+        <v>E77</v>
       </c>
       <c r="B62">
         <v>2016</v>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C62" t="str">
+        <v>B</v>
       </c>
       <c r="D62">
         <v>1411</v>
@@ -1346,18 +1463,14 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>E78</t>
-        </is>
+      <c r="A63" t="str">
+        <v>E78</v>
       </c>
       <c r="B63">
         <v>2018</v>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C63" t="str">
+        <v>C</v>
       </c>
       <c r="D63">
         <v>1484</v>
@@ -1367,18 +1480,14 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>E79</t>
-        </is>
+      <c r="A64" t="str">
+        <v>E79</v>
       </c>
       <c r="B64">
         <v>2019</v>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C64" t="str">
+        <v>D</v>
       </c>
       <c r="D64">
         <v>1557</v>
@@ -1388,18 +1497,14 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>E80</t>
-        </is>
+      <c r="A65" t="str">
+        <v>E80</v>
       </c>
       <c r="B65">
         <v>2020</v>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C65" t="str">
+        <v>A</v>
       </c>
       <c r="D65">
         <v>1630</v>
@@ -1409,18 +1514,14 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>E81</t>
-        </is>
+      <c r="A66" t="str">
+        <v>E81</v>
       </c>
       <c r="B66">
         <v>2020</v>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C66" t="str">
+        <v>B</v>
       </c>
       <c r="D66">
         <v>1703</v>
@@ -1430,18 +1531,14 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>E82</t>
-        </is>
+      <c r="A67" t="str">
+        <v>E82</v>
       </c>
       <c r="B67">
         <v>2022</v>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C67" t="str">
+        <v>C</v>
       </c>
       <c r="D67">
         <v>876</v>
@@ -1451,18 +1548,14 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>E83</t>
-        </is>
+      <c r="A68" t="str">
+        <v>E83</v>
       </c>
       <c r="B68">
         <v>2023</v>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+      <c r="C68" t="str">
+        <v>D</v>
       </c>
       <c r="D68">
         <v>949</v>
@@ -1472,18 +1565,14 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>E84</t>
-        </is>
+      <c r="A69" t="str">
+        <v>E84</v>
       </c>
       <c r="B69">
         <v>2024</v>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="C69" t="str">
+        <v>A</v>
       </c>
       <c r="D69">
         <v>1022</v>
@@ -1493,18 +1582,14 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>E85</t>
-        </is>
+      <c r="A70" t="str">
+        <v>E85</v>
       </c>
       <c r="B70">
         <v>2024</v>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="C70" t="str">
+        <v>B</v>
       </c>
       <c r="D70">
         <v>1095</v>
@@ -1514,18 +1599,14 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>E86</t>
-        </is>
+      <c r="A71" t="str">
+        <v>E86</v>
       </c>
       <c r="B71">
         <v>2026</v>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+      <c r="C71" t="str">
+        <v>C</v>
       </c>
       <c r="D71">
         <v>1168</v>
@@ -1536,5 +1617,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E71"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H71"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>